<commit_message>
Part 1 fully done, NEED to test on Lab Machine
</commit_message>
<xml_diff>
--- a/task1 analysis.xlsx
+++ b/task1 analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackw\Documents\Year 3\Image Processing and Computer Vision\Coursework\IPCV-CW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E659AD7E-9E87-4A18-927B-C11314F0D175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA3B94C-DAD0-4188-A9D4-7C053E7C0F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{1CA8E2B1-F973-4115-B040-CFA540DDAA90}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="37">
   <si>
     <t>F1-Score</t>
   </si>
@@ -135,6 +135,18 @@
   </si>
   <si>
     <t>check</t>
+  </si>
+  <si>
+    <t>Best For Hough Space</t>
+  </si>
+  <si>
+    <t>Worst</t>
+  </si>
+  <si>
+    <t>6, 8</t>
+  </si>
+  <si>
+    <t>1, 3, 7</t>
   </si>
 </sst>
 </file>
@@ -249,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -257,7 +269,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -289,7 +300,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>311372</xdr:colOff>
+      <xdr:colOff>316134</xdr:colOff>
       <xdr:row>100</xdr:row>
       <xdr:rowOff>86433</xdr:rowOff>
     </xdr:to>
@@ -333,9 +344,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1337849</xdr:colOff>
+      <xdr:colOff>1342611</xdr:colOff>
       <xdr:row>95</xdr:row>
-      <xdr:rowOff>61581</xdr:rowOff>
+      <xdr:rowOff>66343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -741,7 +752,7 @@
       <c r="M1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" t="s">
         <v>27</v>
       </c>
       <c r="O1" t="s">
@@ -788,10 +799,10 @@
       <c r="M2" s="2">
         <v>0.5</v>
       </c>
-      <c r="N2" s="7">
-        <v>1</v>
-      </c>
-      <c r="O2" s="7">
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
         <v>0.5</v>
       </c>
     </row>
@@ -835,10 +846,10 @@
       <c r="M3" s="2">
         <v>0.66666666666666596</v>
       </c>
-      <c r="N3" s="7">
-        <v>1</v>
-      </c>
-      <c r="O3" s="7">
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
         <v>0.4</v>
       </c>
     </row>
@@ -882,10 +893,10 @@
       <c r="M4" s="2">
         <v>0.66666666666666596</v>
       </c>
-      <c r="N4" s="7">
-        <v>1</v>
-      </c>
-      <c r="O4" s="7">
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
         <v>0.5</v>
       </c>
     </row>
@@ -929,7 +940,7 @@
       <c r="M5" s="2">
         <v>0.33333333333333298</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5">
         <v>0.5</v>
       </c>
       <c r="O5">
@@ -976,7 +987,7 @@
       <c r="M6" s="2">
         <v>1</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6">
         <v>1</v>
       </c>
       <c r="O6">
@@ -1023,7 +1034,7 @@
       <c r="M7" s="2">
         <v>0.33333333333333298</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7">
         <v>0.3</v>
       </c>
       <c r="O7">
@@ -1070,7 +1081,7 @@
       <c r="M8" s="2">
         <v>0</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8">
         <v>0.25</v>
       </c>
       <c r="O8">
@@ -1117,10 +1128,10 @@
       <c r="M9" s="2">
         <v>0</v>
       </c>
-      <c r="N9" s="7">
-        <v>0</v>
-      </c>
-      <c r="O9" s="7">
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
         <v>0</v>
       </c>
     </row>
@@ -1167,7 +1178,7 @@
       <c r="N10">
         <v>0.33333333333333298</v>
       </c>
-      <c r="O10" s="7">
+      <c r="O10">
         <v>0.5</v>
       </c>
     </row>
@@ -1211,7 +1222,7 @@
       <c r="M11" s="2">
         <v>0.66666666666666596</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11">
         <v>0.5</v>
       </c>
       <c r="O11">
@@ -1305,10 +1316,10 @@
       <c r="M13" s="2">
         <v>0</v>
       </c>
-      <c r="N13" s="7">
-        <v>0</v>
-      </c>
-      <c r="O13" s="7">
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
         <v>0</v>
       </c>
     </row>
@@ -1352,7 +1363,7 @@
       <c r="M14" s="2">
         <v>0.22222222222222199</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14">
         <v>0.625</v>
       </c>
       <c r="O14">
@@ -1399,10 +1410,10 @@
       <c r="M15" s="2">
         <v>0</v>
       </c>
-      <c r="N15" s="7">
-        <v>0</v>
-      </c>
-      <c r="O15" s="7">
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
         <v>0</v>
       </c>
     </row>
@@ -1446,7 +1457,7 @@
       <c r="M16" s="2">
         <v>0</v>
       </c>
-      <c r="N16" s="7">
+      <c r="N16">
         <v>1</v>
       </c>
       <c r="O16">
@@ -1493,7 +1504,7 @@
       <c r="M17" s="4">
         <v>1</v>
       </c>
-      <c r="N17" s="7">
+      <c r="N17">
         <v>1</v>
       </c>
       <c r="O17">
@@ -1570,249 +1581,415 @@
       <c r="C22" t="s">
         <v>0</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="8">
-        <v>1</v>
-      </c>
-      <c r="C23" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
+      <c r="B23" s="7">
+        <v>1</v>
+      </c>
+      <c r="C23" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="8">
-        <v>1</v>
-      </c>
-      <c r="C24" s="8">
+      <c r="B24" s="7">
+        <v>1</v>
+      </c>
+      <c r="C24" s="7">
         <v>0.4</v>
       </c>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="8">
-        <v>1</v>
-      </c>
-      <c r="C25" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
+      <c r="B25" s="7">
+        <v>1</v>
+      </c>
+      <c r="C25" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>5</v>
       </c>
-      <c r="B26" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C26" s="8">
+      <c r="B26" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="C26" s="7">
         <v>0.28571400000000002</v>
       </c>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="8">
-        <v>1</v>
-      </c>
-      <c r="C27" s="8">
+      <c r="B27" s="7">
+        <v>1</v>
+      </c>
+      <c r="C27" s="7">
         <v>0.66666700000000001</v>
       </c>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="7">
         <v>0.2</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="7">
         <v>0.25</v>
       </c>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="7">
         <v>0.25</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="7">
         <v>0.28571400000000002</v>
       </c>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="8">
-        <v>0</v>
-      </c>
-      <c r="C30" s="8">
-        <v>0</v>
-      </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="B30" s="7">
+        <v>0</v>
+      </c>
+      <c r="C30" s="7">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>10</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="7">
         <v>0.33333299999999999</v>
       </c>
-      <c r="C31" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
+      <c r="C31" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C32" s="8">
+      <c r="B32" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="C32" s="7">
         <v>0.66666700000000001</v>
       </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="7">
         <v>0.33333299999999999</v>
       </c>
-      <c r="C33" s="8">
+      <c r="C33" s="7">
         <v>0.33333299999999999</v>
       </c>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="8">
-        <v>0</v>
-      </c>
-      <c r="C34" s="8">
-        <v>0</v>
-      </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B34" s="7">
+        <v>0</v>
+      </c>
+      <c r="C34" s="7">
+        <v>0</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="I34" s="7">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>1</v>
+      </c>
+      <c r="K34" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="L34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="7">
         <v>0.625</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="7">
         <v>0.71428599999999998</v>
       </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="I35" s="7">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>1</v>
+      </c>
+      <c r="K35" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="L35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="8">
-        <v>0</v>
-      </c>
-      <c r="C36" s="8">
-        <v>0</v>
-      </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B36" s="7">
+        <v>0</v>
+      </c>
+      <c r="C36" s="7">
+        <v>0</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="I36" s="7">
+        <v>1</v>
+      </c>
+      <c r="J36">
+        <v>1</v>
+      </c>
+      <c r="K36" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="L36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="8">
-        <v>1</v>
-      </c>
-      <c r="C37" s="8">
+      <c r="B37" s="7">
+        <v>1</v>
+      </c>
+      <c r="C37" s="7">
         <v>0.66666700000000001</v>
       </c>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="I37" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37" s="7">
+        <v>0.28571400000000002</v>
+      </c>
+      <c r="L37">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="8">
-        <v>1</v>
-      </c>
-      <c r="C38" s="8">
+      <c r="B38" s="7">
+        <v>1</v>
+      </c>
+      <c r="C38" s="7">
         <v>0.66666700000000001</v>
       </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-    </row>
-    <row r="39" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B39" s="9">
-        <v>0.55260399999999998</v>
-      </c>
-      <c r="C39" s="10">
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="I38" s="7">
+        <v>1</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
+      </c>
+      <c r="K38" s="7">
+        <v>0.66666700000000001</v>
+      </c>
+      <c r="L38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B39" s="8">
+        <f>AVERAGE(B23:B38)</f>
+        <v>0.54635412499999991</v>
+      </c>
+      <c r="C39" s="9">
         <v>0.41004499999999999</v>
       </c>
-      <c r="D39" s="9"/>
-      <c r="E39" s="10"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="D39" s="8">
+        <f>AVERAGE(C23:C38)</f>
+        <v>0.4022321875</v>
+      </c>
+      <c r="E39" s="9"/>
+      <c r="I39" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="J39">
+        <v>0.1</v>
+      </c>
+      <c r="K39" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="L39">
+        <v>0.18181818181818099</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I40" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="J40">
+        <v>0.75</v>
+      </c>
+      <c r="K40" s="7">
+        <v>0.28571400000000002</v>
+      </c>
+      <c r="L40">
+        <v>0.85714285714285698</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I41" s="7">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41" s="7">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I42" s="7">
+        <v>0.33333299999999999</v>
+      </c>
+      <c r="J42">
+        <v>0.44444444444444398</v>
+      </c>
+      <c r="K42" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="L42">
+        <v>0.61538461538461497</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="I43" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="J43">
+        <v>0.5</v>
+      </c>
+      <c r="K43" s="7">
+        <v>0.66666700000000001</v>
+      </c>
+      <c r="L43">
+        <v>0.66666666666666596</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B44" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" t="s">
+        <v>35</v>
+      </c>
+      <c r="I44" s="7">
+        <v>0.33333299999999999</v>
+      </c>
+      <c r="J44">
+        <v>1</v>
+      </c>
+      <c r="K44" s="7">
+        <v>0.33333299999999999</v>
+      </c>
+      <c r="L44">
+        <v>0.85714285714285698</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>2</v>
       </c>
       <c r="B45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="s">
+        <v>34</v>
+      </c>
+      <c r="F45" t="s">
+        <v>36</v>
+      </c>
+      <c r="I45" s="7">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>1</v>
+      </c>
+      <c r="K45" s="7">
+        <v>0</v>
+      </c>
+      <c r="L45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -1822,8 +1999,20 @@
       <c r="C46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="I46" s="7">
+        <v>0.625</v>
+      </c>
+      <c r="J46">
+        <v>0.5</v>
+      </c>
+      <c r="K46" s="7">
+        <v>0.71428599999999998</v>
+      </c>
+      <c r="L46">
+        <v>0.66666666666666596</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -1833,8 +2022,20 @@
       <c r="C47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="I47" s="7">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47" s="7">
+        <v>0</v>
+      </c>
+      <c r="L47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>5</v>
       </c>
@@ -1844,8 +2045,20 @@
       <c r="C48">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="I48" s="7">
+        <v>1</v>
+      </c>
+      <c r="J48">
+        <v>1</v>
+      </c>
+      <c r="K48" s="7">
+        <v>0.66666700000000001</v>
+      </c>
+      <c r="L48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1853,21 +2066,48 @@
         <v>1</v>
       </c>
       <c r="C49">
-        <v>0.66666666666666596</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+      <c r="I49" s="7">
+        <v>1</v>
+      </c>
+      <c r="J49">
+        <v>1</v>
+      </c>
+      <c r="K49" s="7">
+        <v>0.66666700000000001</v>
+      </c>
+      <c r="L49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A50" t="s">
         <v>7</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
+        <v>0.18181818181818099</v>
+      </c>
+      <c r="I50" s="8">
+        <f>AVERAGE(I34:I49)</f>
+        <v>0.54635412499999991</v>
+      </c>
+      <c r="J50">
+        <f>AVERAGE(J34:J49)</f>
+        <v>0.70590277777777777</v>
+      </c>
+      <c r="K50" s="9">
+        <v>0.41004499999999999</v>
+      </c>
+      <c r="L50">
+        <f>AVERAGE(L34:L49)</f>
+        <v>0.72780136530136508</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -1878,7 +2118,7 @@
         <v>0.85714285714285698</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>9</v>
       </c>
@@ -1889,7 +2129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>10</v>
       </c>
@@ -1900,7 +2140,7 @@
         <v>0.61538461538461497</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>11</v>
       </c>
@@ -1911,7 +2151,7 @@
         <v>0.66666666666666596</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -1919,21 +2159,21 @@
         <v>1</v>
       </c>
       <c r="C55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+        <v>0.85714285714285698</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>13</v>
       </c>
       <c r="B56">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C56">
-        <v>0.66666666666666596</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -1944,7 +2184,7 @@
         <v>0.66666666666666596</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>15</v>
       </c>
@@ -1955,7 +2195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>16</v>
       </c>
@@ -1966,25 +2206,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>17</v>
       </c>
       <c r="B60">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C60">
-        <v>0.66666666666666596</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B61">
         <f>AVERAGE(B45:B60)</f>
-        <v>0.57465277777777768</v>
+        <v>0.70590277777777777</v>
       </c>
       <c r="C61">
         <f>AVERAGE(C45:C60)</f>
-        <v>0.60036630036630012</v>
+        <v>0.72780136530136508</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.45">
@@ -2118,10 +2358,10 @@
         <v>13</v>
       </c>
       <c r="B78">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C78">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D78" t="s">
         <v>32</v>
@@ -2174,11 +2414,11 @@
     <row r="83" spans="1:3" x14ac:dyDescent="0.45">
       <c r="B83">
         <f>AVERAGE(B67:B82)</f>
-        <v>0.74340277777777775</v>
+        <v>0.77465277777777775</v>
       </c>
       <c r="C83">
         <f>AVERAGE(C67:C82)</f>
-        <v>0.78994963369963356</v>
+        <v>0.82119963369963356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>